<commit_message>
Updates for new villages in Ghana North and a few others
</commit_message>
<xml_diff>
--- a/TBM Organization Parameters.xlsx
+++ b/TBM Organization Parameters.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/MicroDrive/SparrowGIT/TBM_Organization_Parameters/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FE922174-C818-3745-9266-4E1D3CA987CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F591CBA-E276-8E47-9A8D-9C611461A0B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="20420" tabRatio="813" firstSheet="18" activeTab="18" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="20420" tabRatio="813" firstSheet="22" activeTab="25" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="TBM" sheetId="7" r:id="rId1"/>
@@ -54,13 +54,15 @@
     <sheet name="WiFi_Languages" sheetId="33" state="hidden" r:id="rId39"/>
     <sheet name="IPMRP" sheetId="45" r:id="rId40"/>
     <sheet name="IPMRN" sheetId="46" r:id="rId41"/>
-    <sheet name="Wifi_Materials" sheetId="37" r:id="rId42"/>
-    <sheet name="Wifi_Downloads" sheetId="38" r:id="rId43"/>
-    <sheet name="Validation" sheetId="34" state="hidden" r:id="rId44"/>
-    <sheet name="Data Valid" sheetId="2" state="hidden" r:id="rId45"/>
+    <sheet name="PMGPE" sheetId="56" r:id="rId42"/>
+    <sheet name="PMGPW" sheetId="57" r:id="rId43"/>
+    <sheet name="Wifi_Materials" sheetId="37" r:id="rId44"/>
+    <sheet name="Wifi_Downloads" sheetId="38" r:id="rId45"/>
+    <sheet name="Validation" sheetId="34" state="hidden" r:id="rId46"/>
+    <sheet name="Data Valid" sheetId="2" state="hidden" r:id="rId47"/>
   </sheets>
   <externalReferences>
-    <externalReference r:id="rId46"/>
+    <externalReference r:id="rId48"/>
   </externalReferences>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="38" hidden="1">WiFi_Languages!$A$1:$D$636</definedName>
@@ -100,7 +102,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4923" uniqueCount="1317">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4985" uniqueCount="1333">
   <si>
     <t>Latitude</t>
   </si>
@@ -4052,19 +4054,74 @@
   </si>
   <si>
     <t>TBM, TBMAR, TBMCV, TBMKA, TBMK, TBMPB, TBMKB, TBMSL, TBMGN, TBMSA, TBMKN, TBMPM</t>
+  </si>
+  <si>
+    <t>Pioneer Mission Global - East Pokot</t>
+  </si>
+  <si>
+    <t>Tangulbei</t>
+  </si>
+  <si>
+    <t>Chemolingot</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pokot </t>
+  </si>
+  <si>
+    <t>Luyha</t>
+  </si>
+  <si>
+    <t>Dholuo</t>
+  </si>
+  <si>
+    <t>Gikuyu</t>
+  </si>
+  <si>
+    <t>Pioneer Mission Global - West Pokot</t>
+  </si>
+  <si>
+    <t>Serewo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mohifong </t>
+  </si>
+  <si>
+    <t>Nakohigu fong</t>
+  </si>
+  <si>
+    <t>Nayili fong North</t>
+  </si>
+  <si>
+    <t>Nayili fong South</t>
+  </si>
+  <si>
+    <t>Kalli fong</t>
+  </si>
+  <si>
+    <t>Kpatuli fong</t>
+  </si>
+  <si>
+    <t>Kuga fong</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="38" x14ac:knownFonts="1">
+  <fonts count="39" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <charset val="129"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -4357,112 +4414,112 @@
   </borders>
   <cellStyleXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="55">
+  <cellXfs count="57">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="16" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="2"/>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="2" applyAlignment="1">
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="2"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="2" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="2" applyFont="1"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="2" applyFont="1"/>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="31" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1"/>
+    <xf numFmtId="16" fontId="31" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="30" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1"/>
-    <xf numFmtId="16" fontId="30" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="0" xfId="2" applyFont="1"/>
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="37" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="33" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="33" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="0" borderId="0" xfId="2" applyFont="1"/>
-    <xf numFmtId="0" fontId="34" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="36" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="36" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="38" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="32" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="37" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -4472,9 +4529,11 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="2" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="14">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -7004,7 +7063,7 @@
   <mergeCells count="1">
     <mergeCell ref="B1:E1"/>
   </mergeCells>
-  <phoneticPr fontId="21" type="noConversion"/>
+  <phoneticPr fontId="22" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
@@ -10071,7 +10130,7 @@
 
 <file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9796B9BC-A579-4EDE-99EB-40D54CC290A0}">
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:E13"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="13" bestFit="1" customWidth="1"/>
@@ -10107,8 +10166,8 @@
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A3" s="22" t="s">
-        <v>1212</v>
+      <c r="A3" s="11" t="s">
+        <v>1330</v>
       </c>
       <c r="B3" t="s">
         <v>117</v>
@@ -10124,8 +10183,8 @@
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A4" s="18" t="s">
-        <v>1213</v>
+      <c r="A4" s="11" t="s">
+        <v>1331</v>
       </c>
       <c r="B4" s="3"/>
       <c r="D4" s="18"/>
@@ -10134,8 +10193,8 @@
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A5" s="18" t="s">
-        <v>1214</v>
+      <c r="A5" s="11" t="s">
+        <v>1332</v>
       </c>
       <c r="B5" s="3"/>
       <c r="D5" s="18"/>
@@ -10144,26 +10203,57 @@
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A6" s="18" t="s">
-        <v>1215</v>
+      <c r="A6" s="11" t="s">
+        <v>1326</v>
       </c>
       <c r="B6" s="2"/>
       <c r="D6" s="18"/>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A7" s="18"/>
+      <c r="A7" s="11" t="s">
+        <v>1327</v>
+      </c>
       <c r="B7" s="3"/>
       <c r="D7" s="4"/>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A8" s="11" t="s">
+        <v>1328</v>
+      </c>
       <c r="B8" s="3"/>
       <c r="D8" s="4"/>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A9" s="11" t="s">
+        <v>1329</v>
+      </c>
       <c r="B9" s="3"/>
       <c r="D9" s="4"/>
     </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A10" s="22" t="s">
+        <v>1212</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A11" s="18" t="s">
+        <v>1213</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A12" s="18" t="s">
+        <v>1214</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A13" s="18" t="s">
+        <v>1215</v>
+      </c>
+    </row>
   </sheetData>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A3:A13">
+    <sortCondition ref="A3:A13"/>
+  </sortState>
   <mergeCells count="1">
     <mergeCell ref="B1:E1"/>
   </mergeCells>
@@ -10175,7 +10265,7 @@
           <x14:formula1>
             <xm:f>Validation!$B$1:$B$5</xm:f>
           </x14:formula1>
-          <xm:sqref>E4:E1048576 E3</xm:sqref>
+          <xm:sqref>E3:E1048576</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -21901,7 +21991,7 @@
   <mergeCells count="1">
     <mergeCell ref="B1:E1"/>
   </mergeCells>
-  <phoneticPr fontId="21" type="noConversion"/>
+  <phoneticPr fontId="22" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
@@ -22194,6 +22284,293 @@
 </file>
 
 <file path=xl/worksheets/sheet42.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{395B706A-E337-434F-B496-90FED3D131D8}">
+  <dimension ref="A1:G15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="22.6640625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A1" s="19" t="s">
+        <v>390</v>
+      </c>
+      <c r="B1" s="51" t="s">
+        <v>1317</v>
+      </c>
+      <c r="C1" s="51"/>
+      <c r="D1" s="51"/>
+      <c r="E1" s="51"/>
+      <c r="F1" s="19" t="s">
+        <v>495</v>
+      </c>
+      <c r="G1" t="s">
+        <v>496</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A2" s="19" t="s">
+        <v>27</v>
+      </c>
+      <c r="B2" s="19" t="s">
+        <v>33</v>
+      </c>
+      <c r="C2" s="19" t="s">
+        <v>69</v>
+      </c>
+      <c r="D2" s="19" t="s">
+        <v>102</v>
+      </c>
+      <c r="E2" s="19" t="s">
+        <v>406</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>1318</v>
+      </c>
+      <c r="B3" t="s">
+        <v>117</v>
+      </c>
+      <c r="C3" t="s">
+        <v>1320</v>
+      </c>
+      <c r="D3" s="55" t="s">
+        <v>505</v>
+      </c>
+      <c r="E3" t="s">
+        <v>407</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>1319</v>
+      </c>
+      <c r="B4" s="3"/>
+      <c r="C4" t="s">
+        <v>471</v>
+      </c>
+      <c r="D4" t="s">
+        <v>471</v>
+      </c>
+      <c r="E4" t="s">
+        <v>408</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B5" s="3"/>
+      <c r="C5" t="s">
+        <v>478</v>
+      </c>
+      <c r="D5" s="55" t="s">
+        <v>478</v>
+      </c>
+      <c r="E5" t="s">
+        <v>409</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B6" s="2"/>
+      <c r="C6" t="s">
+        <v>1321</v>
+      </c>
+      <c r="D6" t="s">
+        <v>1321</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B7" s="3"/>
+      <c r="C7" t="s">
+        <v>468</v>
+      </c>
+      <c r="D7" s="55" t="s">
+        <v>1322</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B8" s="3"/>
+      <c r="C8" t="s">
+        <v>341</v>
+      </c>
+      <c r="D8" s="56" t="s">
+        <v>1323</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B9" s="3"/>
+      <c r="C9" t="s">
+        <v>28</v>
+      </c>
+      <c r="D9" s="56" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B10" s="3"/>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B11" s="3"/>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B12" s="3"/>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B13" s="2"/>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B14" s="3"/>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B15" s="3"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="B1:E1"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet43.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8E4F7BD4-E599-3A48-912C-5B28C4454E56}">
+  <dimension ref="A1:G15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="22.6640625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A1" s="19" t="s">
+        <v>390</v>
+      </c>
+      <c r="B1" s="51" t="s">
+        <v>1324</v>
+      </c>
+      <c r="C1" s="51"/>
+      <c r="D1" s="51"/>
+      <c r="E1" s="51"/>
+      <c r="F1" s="19" t="s">
+        <v>495</v>
+      </c>
+      <c r="G1" t="s">
+        <v>496</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A2" s="19" t="s">
+        <v>27</v>
+      </c>
+      <c r="B2" s="19" t="s">
+        <v>33</v>
+      </c>
+      <c r="C2" s="19" t="s">
+        <v>69</v>
+      </c>
+      <c r="D2" s="19" t="s">
+        <v>102</v>
+      </c>
+      <c r="E2" s="19" t="s">
+        <v>406</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>1325</v>
+      </c>
+      <c r="B3" t="s">
+        <v>117</v>
+      </c>
+      <c r="C3" t="s">
+        <v>1320</v>
+      </c>
+      <c r="D3" s="55" t="s">
+        <v>505</v>
+      </c>
+      <c r="E3" t="s">
+        <v>407</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B4" s="3"/>
+      <c r="C4" t="s">
+        <v>478</v>
+      </c>
+      <c r="D4" s="55" t="s">
+        <v>478</v>
+      </c>
+      <c r="E4" t="s">
+        <v>408</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B5" s="3"/>
+      <c r="C5" t="s">
+        <v>1321</v>
+      </c>
+      <c r="D5" t="s">
+        <v>1321</v>
+      </c>
+      <c r="E5" t="s">
+        <v>409</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B6" s="2"/>
+      <c r="C6" t="s">
+        <v>468</v>
+      </c>
+      <c r="D6" s="55" t="s">
+        <v>1322</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B7" s="3"/>
+      <c r="C7" t="s">
+        <v>341</v>
+      </c>
+      <c r="D7" s="56" t="s">
+        <v>1323</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B8" s="3"/>
+      <c r="C8" t="s">
+        <v>28</v>
+      </c>
+      <c r="D8" s="56" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B9" s="3"/>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B10" s="3"/>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B11" s="3"/>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B12" s="3"/>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B13" s="2"/>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B14" s="3"/>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B15" s="3"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="B1:E1"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet44.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AD4090C0-81F3-488A-BFE0-128FBADFA632}">
   <dimension ref="A1:C13"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -22351,7 +22728,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet43.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet45.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9B17A051-E04F-4C5E-BBD2-8BC11DFBB7DE}">
   <dimension ref="A1:C211"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -24673,7 +25050,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet44.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet46.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EC0388E7-6D7C-494A-B5B0-A06D9161366A}">
   <dimension ref="A1:B5"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -24727,7 +25104,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet45.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet47.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:B25"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -26014,20 +26391,20 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="d75e0231-c5c8-4c84-8215-b760034bdfa5" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
   <Edit>DocumentLibraryForm</Edit>
   <New>DocumentLibraryForm</New>
 </FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="d75e0231-c5c8-4c84-8215-b760034bdfa5" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -26050,6 +26427,14 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F41548EA-A522-4942-9ABF-935FDE65872B}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B09A22F1-B742-4DEC-998C-03DEA5FA7C76}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
@@ -26064,12 +26449,4 @@
     <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F41548EA-A522-4942-9ABF-935FDE65872B}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Add new village to TBMPM
</commit_message>
<xml_diff>
--- a/TBM Organization Parameters.xlsx
+++ b/TBM Organization Parameters.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10531"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10621"/>
   <workbookPr showInkAnnotation="0" autoCompressPictures="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/MicroDrive/SparrowGIT/TBM_Organization_Parameters/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8134AAC5-2FFF-724B-B926-874643E1E131}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FAB3647F-0B8B-B142-9433-257F25B24AE6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="20420" tabRatio="813" firstSheet="7" activeTab="20" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="20420" tabRatio="813" firstSheet="6" activeTab="18" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="TBM" sheetId="7" r:id="rId1"/>
@@ -105,7 +105,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5028" uniqueCount="1352">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5029" uniqueCount="1353">
   <si>
     <t>Latitude</t>
   </si>
@@ -4162,6 +4162,9 @@
   </si>
   <si>
     <t>Lázaro Cárdenas</t>
+  </si>
+  <si>
+    <t>Bangkers</t>
   </si>
 </sst>
 </file>
@@ -4584,13 +4587,13 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="2" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -7931,6 +7934,9 @@
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A5" s="40" t="s">
+        <v>1352</v>
+      </c>
       <c r="C5" s="50" t="s">
         <v>1312</v>
       </c>
@@ -8147,12 +8153,12 @@
       <c r="A1" s="19" t="s">
         <v>390</v>
       </c>
-      <c r="B1" s="55" t="s">
+      <c r="B1" s="53" t="s">
         <v>1017</v>
       </c>
-      <c r="C1" s="55"/>
-      <c r="D1" s="55"/>
-      <c r="E1" s="55"/>
+      <c r="C1" s="53"/>
+      <c r="D1" s="53"/>
+      <c r="E1" s="53"/>
       <c r="F1" s="19" t="s">
         <v>495</v>
       </c>
@@ -8333,12 +8339,12 @@
       <c r="A1" s="19" t="s">
         <v>390</v>
       </c>
-      <c r="B1" s="55" t="s">
+      <c r="B1" s="53" t="s">
         <v>1343</v>
       </c>
-      <c r="C1" s="55"/>
-      <c r="D1" s="55"/>
-      <c r="E1" s="55"/>
+      <c r="C1" s="53"/>
+      <c r="D1" s="53"/>
+      <c r="E1" s="53"/>
       <c r="F1" s="19" t="s">
         <v>495</v>
       </c>
@@ -8448,12 +8454,12 @@
       <c r="A1" s="19" t="s">
         <v>390</v>
       </c>
-      <c r="B1" s="55" t="s">
+      <c r="B1" s="53" t="s">
         <v>1048</v>
       </c>
-      <c r="C1" s="55"/>
-      <c r="D1" s="55"/>
-      <c r="E1" s="55"/>
+      <c r="C1" s="53"/>
+      <c r="D1" s="53"/>
+      <c r="E1" s="53"/>
       <c r="F1" s="19" t="s">
         <v>495</v>
       </c>
@@ -9484,12 +9490,12 @@
       <c r="A1" s="19" t="s">
         <v>390</v>
       </c>
-      <c r="B1" s="53" t="s">
+      <c r="B1" s="55" t="s">
         <v>405</v>
       </c>
-      <c r="C1" s="53"/>
-      <c r="D1" s="53"/>
-      <c r="E1" s="53"/>
+      <c r="C1" s="55"/>
+      <c r="D1" s="55"/>
+      <c r="E1" s="55"/>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A2" s="19" t="s">
@@ -25619,12 +25625,12 @@
       <c r="A1" s="19" t="s">
         <v>390</v>
       </c>
-      <c r="B1" s="55" t="s">
+      <c r="B1" s="53" t="s">
         <v>1167</v>
       </c>
-      <c r="C1" s="55"/>
-      <c r="D1" s="55"/>
-      <c r="E1" s="55"/>
+      <c r="C1" s="53"/>
+      <c r="D1" s="53"/>
+      <c r="E1" s="53"/>
       <c r="F1" s="19" t="s">
         <v>495</v>
       </c>
@@ -25993,12 +25999,12 @@
       <c r="A1" s="19" t="s">
         <v>390</v>
       </c>
-      <c r="B1" s="53" t="s">
+      <c r="B1" s="55" t="s">
         <v>887</v>
       </c>
-      <c r="C1" s="53"/>
-      <c r="D1" s="53"/>
-      <c r="E1" s="53"/>
+      <c r="C1" s="55"/>
+      <c r="D1" s="55"/>
+      <c r="E1" s="55"/>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A2" s="19" t="s">
@@ -26495,15 +26501,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100D3C69E808006664F9CCA3D9BC71AC55D" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="b5845cacad74656bcde11e00306ad31f">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="d75e0231-c5c8-4c84-8215-b760034bdfa5" xmlns:ns4="621de0e2-4b56-4c44-bb0f-ce9b0aec4994" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="2cb8dbf20762a8ba415eee6dfba6bc92" ns3:_="" ns4:_="">
     <xsd:import namespace="d75e0231-c5c8-4c84-8215-b760034bdfa5"/>
@@ -26756,7 +26753,7 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <_activity xmlns="d75e0231-c5c8-4c84-8215-b760034bdfa5" xsi:nil="true"/>
@@ -26764,15 +26761,16 @@
 </p:properties>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F41548EA-A522-4942-9ABF-935FDE65872B}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3B426DB6-4B6A-4971-948B-870FFF62E8F5}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -26791,7 +26789,7 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B09A22F1-B742-4DEC-998C-03DEA5FA7C76}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
@@ -26806,4 +26804,12 @@
     <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F41548EA-A522-4942-9ABF-935FDE65872B}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>